<commit_message>
Auto update histories + intraday analysis
</commit_message>
<xml_diff>
--- a/data/histories/Anguilla history.xlsx
+++ b/data/histories/Anguilla history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3892"/>
+  <dimension ref="A1:E3893"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -105500,6 +105500,33 @@
         </is>
       </c>
     </row>
+    <row r="3893">
+      <c r="A3893" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="B3893" t="inlineStr">
+        <is>
+          <t>Anguila 9PM</t>
+        </is>
+      </c>
+      <c r="C3893" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="D3893" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E3893" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>